<commit_message>
agregados detalles de cada contrato
</commit_message>
<xml_diff>
--- a/backend/TestEjemplo.xlsx
+++ b/backend/TestEjemplo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fiduprevisora-my.sharepoint.com/personal/p_scorrea_fiduprevisora_com_co/Documents/Escritorio/contratos-dashboard/backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="89" documentId="8_{4CA17712-2CC0-4CCD-AA75-F19B91EB8E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CDF8D59-19BE-4331-A348-057C93A6E29B}"/>
+  <xr:revisionPtr revIDLastSave="115" documentId="8_{4CA17712-2CC0-4CCD-AA75-F19B91EB8E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3408718A-4D89-4BB0-A5EC-5D44F2DE8412}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -395,7 +395,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="154">
   <si>
     <t>I.- GENERALIDADES DEL CONTRATO</t>
   </si>
@@ -1084,9 +1084,6 @@
     <t>HOLLMAN ANDRES SUESCUN MENDEZ</t>
   </si>
   <si>
-    <t>DIRECTOR DE SOFTWARE (E )</t>
-  </si>
-  <si>
     <t>FV 3030</t>
   </si>
   <si>
@@ -1111,8 +1108,14 @@
     <t>18 meses</t>
   </si>
   <si>
+    <t>DIRECTORA DE SOFTWARE (E )</t>
+  </si>
+  <si>
+    <t>9 meses</t>
+  </si>
+  <si>
     <r>
-      <t>1-9000-147</t>
+      <t>1-9000-191</t>
     </r>
     <r>
       <rPr>
@@ -2459,7 +2462,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="29" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="415">
+  <cellXfs count="416">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -3509,6 +3512,9 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -3686,7 +3692,7 @@
     <xf numFmtId="15" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="30" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3838,10 +3844,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4247,7 +4249,7 @@
         <v>43</v>
       </c>
       <c r="AO2" s="297">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="AP2" s="298"/>
       <c r="AQ2" s="294">
@@ -4502,7 +4504,7 @@
       <c r="AI7" s="223"/>
       <c r="AJ7" s="223"/>
       <c r="AK7" s="299" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="AL7" s="299"/>
       <c r="AM7" s="299"/>
@@ -4527,7 +4529,7 @@
       <c r="G8" s="223"/>
       <c r="H8" s="223"/>
       <c r="I8" s="279" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J8" s="279"/>
       <c r="K8" s="279"/>
@@ -5639,7 +5641,7 @@
         <v>100</v>
       </c>
       <c r="W28" s="228" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="X28" s="228"/>
       <c r="Y28" s="228"/>
@@ -5708,7 +5710,7 @@
       <c r="U29" s="253"/>
       <c r="V29" s="85"/>
       <c r="W29" s="218" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="X29" s="218"/>
       <c r="Y29" s="218"/>
@@ -5777,7 +5779,7 @@
       <c r="U30" s="253"/>
       <c r="V30" s="85"/>
       <c r="W30" s="218" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="X30" s="218"/>
       <c r="Y30" s="218"/>
@@ -5846,7 +5848,7 @@
       <c r="U31" s="250"/>
       <c r="V31" s="85"/>
       <c r="W31" s="218" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="X31" s="218"/>
       <c r="Y31" s="218"/>
@@ -5971,17 +5973,19 @@
       <c r="V33" s="88" t="s">
         <v>100</v>
       </c>
-      <c r="W33" s="145"/>
+      <c r="W33" s="145" t="s">
+        <v>152</v>
+      </c>
       <c r="X33" s="145"/>
       <c r="Y33" s="145"/>
       <c r="Z33" s="145"/>
       <c r="AA33" s="146"/>
-      <c r="AB33" s="401"/>
+      <c r="AB33" s="402"/>
       <c r="AC33" s="306"/>
       <c r="AD33" s="306"/>
       <c r="AE33" s="306"/>
       <c r="AF33" s="306"/>
-      <c r="AG33" s="402"/>
+      <c r="AG33" s="403"/>
       <c r="AH33" s="316"/>
       <c r="AI33" s="317"/>
       <c r="AJ33" s="317"/>
@@ -6022,7 +6026,7 @@
       <c r="T34" s="2"/>
       <c r="U34" s="2"/>
       <c r="V34" s="2"/>
-      <c r="W34" s="2"/>
+      <c r="W34" s="104"/>
       <c r="X34" s="2"/>
       <c r="Y34" s="2"/>
       <c r="Z34" s="2"/>
@@ -6370,24 +6374,24 @@
       <c r="B41" s="58">
         <v>1</v>
       </c>
-      <c r="C41" s="408">
+      <c r="C41" s="409">
         <v>45924</v>
       </c>
-      <c r="D41" s="409"/>
-      <c r="E41" s="409"/>
-      <c r="F41" s="409"/>
-      <c r="G41" s="409"/>
-      <c r="H41" s="410"/>
-      <c r="I41" s="403">
+      <c r="D41" s="410"/>
+      <c r="E41" s="410"/>
+      <c r="F41" s="410"/>
+      <c r="G41" s="410"/>
+      <c r="H41" s="411"/>
+      <c r="I41" s="404">
         <v>11103</v>
       </c>
-      <c r="J41" s="404"/>
-      <c r="K41" s="404"/>
-      <c r="L41" s="404"/>
-      <c r="M41" s="404"/>
-      <c r="N41" s="404"/>
-      <c r="O41" s="404"/>
-      <c r="P41" s="405"/>
+      <c r="J41" s="405"/>
+      <c r="K41" s="405"/>
+      <c r="L41" s="405"/>
+      <c r="M41" s="405"/>
+      <c r="N41" s="405"/>
+      <c r="O41" s="405"/>
+      <c r="P41" s="406"/>
       <c r="Q41" s="322" t="s">
         <v>109</v>
       </c>
@@ -6431,20 +6435,20 @@
       <c r="B42" s="27">
         <v>2</v>
       </c>
-      <c r="C42" s="411"/>
-      <c r="D42" s="412"/>
-      <c r="E42" s="412"/>
-      <c r="F42" s="412"/>
-      <c r="G42" s="412"/>
-      <c r="H42" s="413"/>
-      <c r="I42" s="406"/>
+      <c r="C42" s="412"/>
+      <c r="D42" s="413"/>
+      <c r="E42" s="413"/>
+      <c r="F42" s="413"/>
+      <c r="G42" s="413"/>
+      <c r="H42" s="414"/>
+      <c r="I42" s="407"/>
       <c r="J42" s="113"/>
       <c r="K42" s="113"/>
       <c r="L42" s="113"/>
       <c r="M42" s="113"/>
       <c r="N42" s="113"/>
       <c r="O42" s="113"/>
-      <c r="P42" s="407"/>
+      <c r="P42" s="408"/>
       <c r="Q42" s="109" t="s">
         <v>111</v>
       </c>
@@ -7646,7 +7650,7 @@
         <v>4</v>
       </c>
       <c r="C64" s="219" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D64" s="137"/>
       <c r="E64" s="137"/>
@@ -7659,7 +7663,7 @@
       <c r="L64" s="137"/>
       <c r="M64" s="137"/>
       <c r="N64" s="172" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="O64" s="173"/>
       <c r="P64" s="173"/>
@@ -7852,53 +7856,53 @@
     </row>
     <row r="68" spans="1:47" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="13"/>
-      <c r="B68" s="414" t="s">
+      <c r="B68" s="355" t="s">
         <v>74</v>
       </c>
-      <c r="C68" s="414"/>
-      <c r="D68" s="414"/>
-      <c r="E68" s="414"/>
-      <c r="F68" s="414"/>
-      <c r="G68" s="414"/>
-      <c r="H68" s="414"/>
-      <c r="I68" s="414"/>
-      <c r="J68" s="414"/>
-      <c r="K68" s="414"/>
-      <c r="L68" s="414"/>
-      <c r="M68" s="414"/>
-      <c r="N68" s="414"/>
-      <c r="O68" s="414"/>
-      <c r="P68" s="414"/>
-      <c r="Q68" s="414"/>
-      <c r="R68" s="414"/>
-      <c r="S68" s="414"/>
-      <c r="T68" s="414"/>
-      <c r="U68" s="414"/>
-      <c r="V68" s="414"/>
-      <c r="W68" s="414"/>
-      <c r="X68" s="414"/>
-      <c r="Y68" s="414"/>
-      <c r="Z68" s="414"/>
-      <c r="AA68" s="414"/>
-      <c r="AB68" s="414"/>
-      <c r="AC68" s="414"/>
-      <c r="AD68" s="414"/>
-      <c r="AE68" s="414"/>
-      <c r="AF68" s="414"/>
-      <c r="AG68" s="414"/>
-      <c r="AH68" s="414"/>
-      <c r="AI68" s="414"/>
-      <c r="AJ68" s="414"/>
-      <c r="AK68" s="414"/>
-      <c r="AL68" s="414"/>
-      <c r="AM68" s="414"/>
-      <c r="AN68" s="414"/>
-      <c r="AO68" s="414"/>
-      <c r="AP68" s="414"/>
-      <c r="AQ68" s="414"/>
-      <c r="AR68" s="414"/>
-      <c r="AS68" s="414"/>
-      <c r="AT68" s="414"/>
+      <c r="C68" s="355"/>
+      <c r="D68" s="355"/>
+      <c r="E68" s="355"/>
+      <c r="F68" s="355"/>
+      <c r="G68" s="355"/>
+      <c r="H68" s="355"/>
+      <c r="I68" s="355"/>
+      <c r="J68" s="355"/>
+      <c r="K68" s="355"/>
+      <c r="L68" s="355"/>
+      <c r="M68" s="355"/>
+      <c r="N68" s="355"/>
+      <c r="O68" s="355"/>
+      <c r="P68" s="355"/>
+      <c r="Q68" s="355"/>
+      <c r="R68" s="355"/>
+      <c r="S68" s="355"/>
+      <c r="T68" s="355"/>
+      <c r="U68" s="355"/>
+      <c r="V68" s="355"/>
+      <c r="W68" s="355"/>
+      <c r="X68" s="355"/>
+      <c r="Y68" s="355"/>
+      <c r="Z68" s="355"/>
+      <c r="AA68" s="355"/>
+      <c r="AB68" s="355"/>
+      <c r="AC68" s="355"/>
+      <c r="AD68" s="355"/>
+      <c r="AE68" s="355"/>
+      <c r="AF68" s="355"/>
+      <c r="AG68" s="355"/>
+      <c r="AH68" s="355"/>
+      <c r="AI68" s="355"/>
+      <c r="AJ68" s="355"/>
+      <c r="AK68" s="355"/>
+      <c r="AL68" s="355"/>
+      <c r="AM68" s="355"/>
+      <c r="AN68" s="355"/>
+      <c r="AO68" s="355"/>
+      <c r="AP68" s="355"/>
+      <c r="AQ68" s="355"/>
+      <c r="AR68" s="355"/>
+      <c r="AS68" s="355"/>
+      <c r="AT68" s="355"/>
       <c r="AU68" s="14"/>
     </row>
     <row r="69" spans="1:47" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -8098,25 +8102,25 @@
       <c r="AA72" s="154"/>
       <c r="AB72" s="154"/>
       <c r="AC72" s="154"/>
-      <c r="AD72" s="359" t="s">
+      <c r="AD72" s="360" t="s">
         <v>137</v>
       </c>
-      <c r="AE72" s="360"/>
-      <c r="AF72" s="361"/>
-      <c r="AG72" s="359"/>
-      <c r="AH72" s="360"/>
-      <c r="AI72" s="361"/>
-      <c r="AJ72" s="362"/>
-      <c r="AK72" s="363"/>
-      <c r="AL72" s="363"/>
-      <c r="AM72" s="363"/>
-      <c r="AN72" s="363"/>
-      <c r="AO72" s="363"/>
-      <c r="AP72" s="363"/>
-      <c r="AQ72" s="363"/>
-      <c r="AR72" s="363"/>
-      <c r="AS72" s="363"/>
-      <c r="AT72" s="364"/>
+      <c r="AE72" s="361"/>
+      <c r="AF72" s="362"/>
+      <c r="AG72" s="360"/>
+      <c r="AH72" s="361"/>
+      <c r="AI72" s="362"/>
+      <c r="AJ72" s="363"/>
+      <c r="AK72" s="364"/>
+      <c r="AL72" s="364"/>
+      <c r="AM72" s="364"/>
+      <c r="AN72" s="364"/>
+      <c r="AO72" s="364"/>
+      <c r="AP72" s="364"/>
+      <c r="AQ72" s="364"/>
+      <c r="AR72" s="364"/>
+      <c r="AS72" s="364"/>
+      <c r="AT72" s="365"/>
       <c r="AU72" s="14"/>
     </row>
     <row r="73" spans="1:47" ht="189" customHeight="1" x14ac:dyDescent="0.35">
@@ -8153,25 +8157,25 @@
       <c r="AA73" s="154"/>
       <c r="AB73" s="154"/>
       <c r="AC73" s="154"/>
-      <c r="AD73" s="359" t="s">
+      <c r="AD73" s="360" t="s">
         <v>137</v>
       </c>
-      <c r="AE73" s="360"/>
-      <c r="AF73" s="361"/>
-      <c r="AG73" s="359"/>
-      <c r="AH73" s="360"/>
-      <c r="AI73" s="361"/>
-      <c r="AJ73" s="362"/>
-      <c r="AK73" s="363"/>
-      <c r="AL73" s="363"/>
-      <c r="AM73" s="363"/>
-      <c r="AN73" s="363"/>
-      <c r="AO73" s="363"/>
-      <c r="AP73" s="363"/>
-      <c r="AQ73" s="363"/>
-      <c r="AR73" s="363"/>
-      <c r="AS73" s="363"/>
-      <c r="AT73" s="364"/>
+      <c r="AE73" s="361"/>
+      <c r="AF73" s="362"/>
+      <c r="AG73" s="360"/>
+      <c r="AH73" s="361"/>
+      <c r="AI73" s="362"/>
+      <c r="AJ73" s="363"/>
+      <c r="AK73" s="364"/>
+      <c r="AL73" s="364"/>
+      <c r="AM73" s="364"/>
+      <c r="AN73" s="364"/>
+      <c r="AO73" s="364"/>
+      <c r="AP73" s="364"/>
+      <c r="AQ73" s="364"/>
+      <c r="AR73" s="364"/>
+      <c r="AS73" s="364"/>
+      <c r="AT73" s="365"/>
       <c r="AU73" s="14"/>
     </row>
     <row r="74" spans="1:47" ht="157" customHeight="1" x14ac:dyDescent="0.35">
@@ -8210,25 +8214,25 @@
       <c r="AA74" s="154"/>
       <c r="AB74" s="154"/>
       <c r="AC74" s="154"/>
-      <c r="AD74" s="359"/>
-      <c r="AE74" s="360"/>
-      <c r="AF74" s="361"/>
-      <c r="AG74" s="359"/>
-      <c r="AH74" s="360"/>
-      <c r="AI74" s="361"/>
-      <c r="AJ74" s="365" t="s">
+      <c r="AD74" s="360"/>
+      <c r="AE74" s="361"/>
+      <c r="AF74" s="362"/>
+      <c r="AG74" s="360"/>
+      <c r="AH74" s="361"/>
+      <c r="AI74" s="362"/>
+      <c r="AJ74" s="366" t="s">
         <v>138</v>
       </c>
-      <c r="AK74" s="366"/>
-      <c r="AL74" s="366"/>
-      <c r="AM74" s="366"/>
-      <c r="AN74" s="366"/>
-      <c r="AO74" s="366"/>
-      <c r="AP74" s="366"/>
-      <c r="AQ74" s="366"/>
-      <c r="AR74" s="366"/>
-      <c r="AS74" s="366"/>
-      <c r="AT74" s="367"/>
+      <c r="AK74" s="367"/>
+      <c r="AL74" s="367"/>
+      <c r="AM74" s="367"/>
+      <c r="AN74" s="367"/>
+      <c r="AO74" s="367"/>
+      <c r="AP74" s="367"/>
+      <c r="AQ74" s="367"/>
+      <c r="AR74" s="367"/>
+      <c r="AS74" s="367"/>
+      <c r="AT74" s="368"/>
       <c r="AU74" s="14"/>
     </row>
     <row r="75" spans="1:47" ht="196.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8267,25 +8271,25 @@
       <c r="AA75" s="154"/>
       <c r="AB75" s="154"/>
       <c r="AC75" s="154"/>
-      <c r="AD75" s="359"/>
-      <c r="AE75" s="360"/>
-      <c r="AF75" s="361"/>
-      <c r="AG75" s="359"/>
-      <c r="AH75" s="360"/>
-      <c r="AI75" s="361"/>
-      <c r="AJ75" s="365" t="s">
+      <c r="AD75" s="360"/>
+      <c r="AE75" s="361"/>
+      <c r="AF75" s="362"/>
+      <c r="AG75" s="360"/>
+      <c r="AH75" s="361"/>
+      <c r="AI75" s="362"/>
+      <c r="AJ75" s="366" t="s">
         <v>139</v>
       </c>
-      <c r="AK75" s="366"/>
-      <c r="AL75" s="366"/>
-      <c r="AM75" s="366"/>
-      <c r="AN75" s="366"/>
-      <c r="AO75" s="366"/>
-      <c r="AP75" s="366"/>
-      <c r="AQ75" s="366"/>
-      <c r="AR75" s="366"/>
-      <c r="AS75" s="366"/>
-      <c r="AT75" s="367"/>
+      <c r="AK75" s="367"/>
+      <c r="AL75" s="367"/>
+      <c r="AM75" s="367"/>
+      <c r="AN75" s="367"/>
+      <c r="AO75" s="367"/>
+      <c r="AP75" s="367"/>
+      <c r="AQ75" s="367"/>
+      <c r="AR75" s="367"/>
+      <c r="AS75" s="367"/>
+      <c r="AT75" s="368"/>
       <c r="AU75" s="14"/>
     </row>
     <row r="76" spans="1:47" ht="41" customHeight="1" x14ac:dyDescent="0.35">
@@ -8322,25 +8326,25 @@
       <c r="AA76" s="154"/>
       <c r="AB76" s="154"/>
       <c r="AC76" s="154"/>
-      <c r="AD76" s="359" t="s">
+      <c r="AD76" s="360" t="s">
         <v>137</v>
       </c>
-      <c r="AE76" s="360"/>
-      <c r="AF76" s="361"/>
-      <c r="AG76" s="359"/>
-      <c r="AH76" s="360"/>
-      <c r="AI76" s="361"/>
-      <c r="AJ76" s="362"/>
-      <c r="AK76" s="363"/>
-      <c r="AL76" s="363"/>
-      <c r="AM76" s="363"/>
-      <c r="AN76" s="363"/>
-      <c r="AO76" s="363"/>
-      <c r="AP76" s="363"/>
-      <c r="AQ76" s="363"/>
-      <c r="AR76" s="363"/>
-      <c r="AS76" s="363"/>
-      <c r="AT76" s="364"/>
+      <c r="AE76" s="361"/>
+      <c r="AF76" s="362"/>
+      <c r="AG76" s="360"/>
+      <c r="AH76" s="361"/>
+      <c r="AI76" s="362"/>
+      <c r="AJ76" s="363"/>
+      <c r="AK76" s="364"/>
+      <c r="AL76" s="364"/>
+      <c r="AM76" s="364"/>
+      <c r="AN76" s="364"/>
+      <c r="AO76" s="364"/>
+      <c r="AP76" s="364"/>
+      <c r="AQ76" s="364"/>
+      <c r="AR76" s="364"/>
+      <c r="AS76" s="364"/>
+      <c r="AT76" s="365"/>
       <c r="AU76" s="14"/>
     </row>
     <row r="77" spans="1:47" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8379,25 +8383,25 @@
       <c r="AA77" s="154"/>
       <c r="AB77" s="154"/>
       <c r="AC77" s="154"/>
-      <c r="AD77" s="359"/>
-      <c r="AE77" s="360"/>
-      <c r="AF77" s="361"/>
-      <c r="AG77" s="359"/>
-      <c r="AH77" s="360"/>
-      <c r="AI77" s="361"/>
-      <c r="AJ77" s="365" t="s">
+      <c r="AD77" s="360"/>
+      <c r="AE77" s="361"/>
+      <c r="AF77" s="362"/>
+      <c r="AG77" s="360"/>
+      <c r="AH77" s="361"/>
+      <c r="AI77" s="362"/>
+      <c r="AJ77" s="366" t="s">
         <v>139</v>
       </c>
-      <c r="AK77" s="366"/>
-      <c r="AL77" s="366"/>
-      <c r="AM77" s="366"/>
-      <c r="AN77" s="366"/>
-      <c r="AO77" s="366"/>
-      <c r="AP77" s="366"/>
-      <c r="AQ77" s="366"/>
-      <c r="AR77" s="366"/>
-      <c r="AS77" s="366"/>
-      <c r="AT77" s="367"/>
+      <c r="AK77" s="367"/>
+      <c r="AL77" s="367"/>
+      <c r="AM77" s="367"/>
+      <c r="AN77" s="367"/>
+      <c r="AO77" s="367"/>
+      <c r="AP77" s="367"/>
+      <c r="AQ77" s="367"/>
+      <c r="AR77" s="367"/>
+      <c r="AS77" s="367"/>
+      <c r="AT77" s="368"/>
       <c r="AU77" s="14"/>
     </row>
     <row r="78" spans="1:47" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -8436,25 +8440,25 @@
       <c r="AA78" s="154"/>
       <c r="AB78" s="154"/>
       <c r="AC78" s="154"/>
-      <c r="AD78" s="359"/>
-      <c r="AE78" s="360"/>
-      <c r="AF78" s="361"/>
-      <c r="AG78" s="359"/>
-      <c r="AH78" s="360"/>
-      <c r="AI78" s="361"/>
-      <c r="AJ78" s="365" t="s">
+      <c r="AD78" s="360"/>
+      <c r="AE78" s="361"/>
+      <c r="AF78" s="362"/>
+      <c r="AG78" s="360"/>
+      <c r="AH78" s="361"/>
+      <c r="AI78" s="362"/>
+      <c r="AJ78" s="366" t="s">
         <v>139</v>
       </c>
-      <c r="AK78" s="366"/>
-      <c r="AL78" s="366"/>
-      <c r="AM78" s="366"/>
-      <c r="AN78" s="366"/>
-      <c r="AO78" s="366"/>
-      <c r="AP78" s="366"/>
-      <c r="AQ78" s="366"/>
-      <c r="AR78" s="366"/>
-      <c r="AS78" s="366"/>
-      <c r="AT78" s="367"/>
+      <c r="AK78" s="367"/>
+      <c r="AL78" s="367"/>
+      <c r="AM78" s="367"/>
+      <c r="AN78" s="367"/>
+      <c r="AO78" s="367"/>
+      <c r="AP78" s="367"/>
+      <c r="AQ78" s="367"/>
+      <c r="AR78" s="367"/>
+      <c r="AS78" s="367"/>
+      <c r="AT78" s="368"/>
       <c r="AU78" s="14"/>
     </row>
     <row r="79" spans="1:47" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -8491,25 +8495,25 @@
       <c r="AA79" s="154"/>
       <c r="AB79" s="154"/>
       <c r="AC79" s="154"/>
-      <c r="AD79" s="359" t="s">
+      <c r="AD79" s="360" t="s">
         <v>137</v>
       </c>
-      <c r="AE79" s="360"/>
-      <c r="AF79" s="361"/>
-      <c r="AG79" s="359"/>
-      <c r="AH79" s="360"/>
-      <c r="AI79" s="361"/>
-      <c r="AJ79" s="362"/>
-      <c r="AK79" s="363"/>
-      <c r="AL79" s="363"/>
-      <c r="AM79" s="363"/>
-      <c r="AN79" s="363"/>
-      <c r="AO79" s="363"/>
-      <c r="AP79" s="363"/>
-      <c r="AQ79" s="363"/>
-      <c r="AR79" s="363"/>
-      <c r="AS79" s="363"/>
-      <c r="AT79" s="364"/>
+      <c r="AE79" s="361"/>
+      <c r="AF79" s="362"/>
+      <c r="AG79" s="360"/>
+      <c r="AH79" s="361"/>
+      <c r="AI79" s="362"/>
+      <c r="AJ79" s="363"/>
+      <c r="AK79" s="364"/>
+      <c r="AL79" s="364"/>
+      <c r="AM79" s="364"/>
+      <c r="AN79" s="364"/>
+      <c r="AO79" s="364"/>
+      <c r="AP79" s="364"/>
+      <c r="AQ79" s="364"/>
+      <c r="AR79" s="364"/>
+      <c r="AS79" s="364"/>
+      <c r="AT79" s="365"/>
       <c r="AU79" s="14"/>
     </row>
     <row r="80" spans="1:47" ht="38" customHeight="1" x14ac:dyDescent="0.35">
@@ -8548,25 +8552,25 @@
       </c>
       <c r="AB80" s="154"/>
       <c r="AC80" s="154"/>
-      <c r="AD80" s="359"/>
-      <c r="AE80" s="360"/>
-      <c r="AF80" s="361"/>
-      <c r="AG80" s="359"/>
-      <c r="AH80" s="360"/>
-      <c r="AI80" s="361"/>
-      <c r="AJ80" s="365" t="s">
+      <c r="AD80" s="360"/>
+      <c r="AE80" s="361"/>
+      <c r="AF80" s="362"/>
+      <c r="AG80" s="360"/>
+      <c r="AH80" s="361"/>
+      <c r="AI80" s="362"/>
+      <c r="AJ80" s="366" t="s">
         <v>139</v>
       </c>
-      <c r="AK80" s="366"/>
-      <c r="AL80" s="366"/>
-      <c r="AM80" s="366"/>
-      <c r="AN80" s="366"/>
-      <c r="AO80" s="366"/>
-      <c r="AP80" s="366"/>
-      <c r="AQ80" s="366"/>
-      <c r="AR80" s="366"/>
-      <c r="AS80" s="366"/>
-      <c r="AT80" s="367"/>
+      <c r="AK80" s="367"/>
+      <c r="AL80" s="367"/>
+      <c r="AM80" s="367"/>
+      <c r="AN80" s="367"/>
+      <c r="AO80" s="367"/>
+      <c r="AP80" s="367"/>
+      <c r="AQ80" s="367"/>
+      <c r="AR80" s="367"/>
+      <c r="AS80" s="367"/>
+      <c r="AT80" s="368"/>
       <c r="AU80" s="14"/>
     </row>
     <row r="81" spans="1:47" ht="26" customHeight="1" x14ac:dyDescent="0.35">
@@ -8605,25 +8609,25 @@
       </c>
       <c r="AB81" s="154"/>
       <c r="AC81" s="154"/>
-      <c r="AD81" s="359"/>
-      <c r="AE81" s="360"/>
-      <c r="AF81" s="361"/>
-      <c r="AG81" s="359"/>
-      <c r="AH81" s="360"/>
-      <c r="AI81" s="361"/>
-      <c r="AJ81" s="365" t="s">
+      <c r="AD81" s="360"/>
+      <c r="AE81" s="361"/>
+      <c r="AF81" s="362"/>
+      <c r="AG81" s="360"/>
+      <c r="AH81" s="361"/>
+      <c r="AI81" s="362"/>
+      <c r="AJ81" s="366" t="s">
         <v>139</v>
       </c>
-      <c r="AK81" s="366"/>
-      <c r="AL81" s="366"/>
-      <c r="AM81" s="366"/>
-      <c r="AN81" s="366"/>
-      <c r="AO81" s="366"/>
-      <c r="AP81" s="366"/>
-      <c r="AQ81" s="366"/>
-      <c r="AR81" s="366"/>
-      <c r="AS81" s="366"/>
-      <c r="AT81" s="367"/>
+      <c r="AK81" s="367"/>
+      <c r="AL81" s="367"/>
+      <c r="AM81" s="367"/>
+      <c r="AN81" s="367"/>
+      <c r="AO81" s="367"/>
+      <c r="AP81" s="367"/>
+      <c r="AQ81" s="367"/>
+      <c r="AR81" s="367"/>
+      <c r="AS81" s="367"/>
+      <c r="AT81" s="368"/>
       <c r="AU81" s="14"/>
     </row>
     <row r="82" spans="1:47" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8662,25 +8666,25 @@
       </c>
       <c r="AB82" s="154"/>
       <c r="AC82" s="154"/>
-      <c r="AD82" s="359"/>
-      <c r="AE82" s="360"/>
-      <c r="AF82" s="361"/>
-      <c r="AG82" s="359"/>
-      <c r="AH82" s="360"/>
-      <c r="AI82" s="361"/>
-      <c r="AJ82" s="365" t="s">
+      <c r="AD82" s="360"/>
+      <c r="AE82" s="361"/>
+      <c r="AF82" s="362"/>
+      <c r="AG82" s="360"/>
+      <c r="AH82" s="361"/>
+      <c r="AI82" s="362"/>
+      <c r="AJ82" s="366" t="s">
         <v>139</v>
       </c>
-      <c r="AK82" s="366"/>
-      <c r="AL82" s="366"/>
-      <c r="AM82" s="366"/>
-      <c r="AN82" s="366"/>
-      <c r="AO82" s="366"/>
-      <c r="AP82" s="366"/>
-      <c r="AQ82" s="366"/>
-      <c r="AR82" s="366"/>
-      <c r="AS82" s="366"/>
-      <c r="AT82" s="367"/>
+      <c r="AK82" s="367"/>
+      <c r="AL82" s="367"/>
+      <c r="AM82" s="367"/>
+      <c r="AN82" s="367"/>
+      <c r="AO82" s="367"/>
+      <c r="AP82" s="367"/>
+      <c r="AQ82" s="367"/>
+      <c r="AR82" s="367"/>
+      <c r="AS82" s="367"/>
+      <c r="AT82" s="368"/>
       <c r="AU82" s="14"/>
     </row>
     <row r="83" spans="1:47" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -8717,25 +8721,25 @@
       <c r="AA83" s="154"/>
       <c r="AB83" s="154"/>
       <c r="AC83" s="154"/>
-      <c r="AD83" s="359" t="s">
+      <c r="AD83" s="360" t="s">
         <v>137</v>
       </c>
-      <c r="AE83" s="360"/>
-      <c r="AF83" s="361"/>
-      <c r="AG83" s="359"/>
-      <c r="AH83" s="360"/>
-      <c r="AI83" s="361"/>
-      <c r="AJ83" s="362"/>
-      <c r="AK83" s="363"/>
-      <c r="AL83" s="363"/>
-      <c r="AM83" s="363"/>
-      <c r="AN83" s="363"/>
-      <c r="AO83" s="363"/>
-      <c r="AP83" s="363"/>
-      <c r="AQ83" s="363"/>
-      <c r="AR83" s="363"/>
-      <c r="AS83" s="363"/>
-      <c r="AT83" s="364"/>
+      <c r="AE83" s="361"/>
+      <c r="AF83" s="362"/>
+      <c r="AG83" s="360"/>
+      <c r="AH83" s="361"/>
+      <c r="AI83" s="362"/>
+      <c r="AJ83" s="363"/>
+      <c r="AK83" s="364"/>
+      <c r="AL83" s="364"/>
+      <c r="AM83" s="364"/>
+      <c r="AN83" s="364"/>
+      <c r="AO83" s="364"/>
+      <c r="AP83" s="364"/>
+      <c r="AQ83" s="364"/>
+      <c r="AR83" s="364"/>
+      <c r="AS83" s="364"/>
+      <c r="AT83" s="365"/>
       <c r="AU83" s="14"/>
     </row>
     <row r="84" spans="1:47" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -8772,25 +8776,25 @@
       <c r="AA84" s="154"/>
       <c r="AB84" s="154"/>
       <c r="AC84" s="154"/>
-      <c r="AD84" s="359" t="s">
+      <c r="AD84" s="360" t="s">
         <v>137</v>
       </c>
-      <c r="AE84" s="360"/>
-      <c r="AF84" s="361"/>
-      <c r="AG84" s="359"/>
-      <c r="AH84" s="360"/>
-      <c r="AI84" s="361"/>
-      <c r="AJ84" s="362"/>
-      <c r="AK84" s="363"/>
-      <c r="AL84" s="363"/>
-      <c r="AM84" s="363"/>
-      <c r="AN84" s="363"/>
-      <c r="AO84" s="363"/>
-      <c r="AP84" s="363"/>
-      <c r="AQ84" s="363"/>
-      <c r="AR84" s="363"/>
-      <c r="AS84" s="363"/>
-      <c r="AT84" s="364"/>
+      <c r="AE84" s="361"/>
+      <c r="AF84" s="362"/>
+      <c r="AG84" s="360"/>
+      <c r="AH84" s="361"/>
+      <c r="AI84" s="362"/>
+      <c r="AJ84" s="363"/>
+      <c r="AK84" s="364"/>
+      <c r="AL84" s="364"/>
+      <c r="AM84" s="364"/>
+      <c r="AN84" s="364"/>
+      <c r="AO84" s="364"/>
+      <c r="AP84" s="364"/>
+      <c r="AQ84" s="364"/>
+      <c r="AR84" s="364"/>
+      <c r="AS84" s="364"/>
+      <c r="AT84" s="365"/>
       <c r="AU84" s="14"/>
     </row>
     <row r="85" spans="1:47" ht="45.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8827,25 +8831,25 @@
       <c r="AA85" s="154"/>
       <c r="AB85" s="154"/>
       <c r="AC85" s="154"/>
-      <c r="AD85" s="359" t="s">
+      <c r="AD85" s="360" t="s">
         <v>137</v>
       </c>
-      <c r="AE85" s="360"/>
-      <c r="AF85" s="361"/>
-      <c r="AG85" s="359"/>
-      <c r="AH85" s="360"/>
-      <c r="AI85" s="361"/>
-      <c r="AJ85" s="362"/>
-      <c r="AK85" s="363"/>
-      <c r="AL85" s="363"/>
-      <c r="AM85" s="363"/>
-      <c r="AN85" s="363"/>
-      <c r="AO85" s="363"/>
-      <c r="AP85" s="363"/>
-      <c r="AQ85" s="363"/>
-      <c r="AR85" s="363"/>
-      <c r="AS85" s="363"/>
-      <c r="AT85" s="364"/>
+      <c r="AE85" s="361"/>
+      <c r="AF85" s="362"/>
+      <c r="AG85" s="360"/>
+      <c r="AH85" s="361"/>
+      <c r="AI85" s="362"/>
+      <c r="AJ85" s="363"/>
+      <c r="AK85" s="364"/>
+      <c r="AL85" s="364"/>
+      <c r="AM85" s="364"/>
+      <c r="AN85" s="364"/>
+      <c r="AO85" s="364"/>
+      <c r="AP85" s="364"/>
+      <c r="AQ85" s="364"/>
+      <c r="AR85" s="364"/>
+      <c r="AS85" s="364"/>
+      <c r="AT85" s="365"/>
       <c r="AU85" s="14"/>
     </row>
     <row r="86" spans="1:47" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -8882,25 +8886,25 @@
       <c r="AA86" s="154"/>
       <c r="AB86" s="154"/>
       <c r="AC86" s="154"/>
-      <c r="AD86" s="359" t="s">
+      <c r="AD86" s="360" t="s">
         <v>137</v>
       </c>
-      <c r="AE86" s="360"/>
-      <c r="AF86" s="361"/>
-      <c r="AG86" s="359"/>
-      <c r="AH86" s="360"/>
-      <c r="AI86" s="361"/>
-      <c r="AJ86" s="362"/>
-      <c r="AK86" s="363"/>
-      <c r="AL86" s="363"/>
-      <c r="AM86" s="363"/>
-      <c r="AN86" s="363"/>
-      <c r="AO86" s="363"/>
-      <c r="AP86" s="363"/>
-      <c r="AQ86" s="363"/>
-      <c r="AR86" s="363"/>
-      <c r="AS86" s="363"/>
-      <c r="AT86" s="364"/>
+      <c r="AE86" s="361"/>
+      <c r="AF86" s="362"/>
+      <c r="AG86" s="360"/>
+      <c r="AH86" s="361"/>
+      <c r="AI86" s="362"/>
+      <c r="AJ86" s="363"/>
+      <c r="AK86" s="364"/>
+      <c r="AL86" s="364"/>
+      <c r="AM86" s="364"/>
+      <c r="AN86" s="364"/>
+      <c r="AO86" s="364"/>
+      <c r="AP86" s="364"/>
+      <c r="AQ86" s="364"/>
+      <c r="AR86" s="364"/>
+      <c r="AS86" s="364"/>
+      <c r="AT86" s="365"/>
       <c r="AU86" s="14"/>
     </row>
     <row r="87" spans="1:47" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -8937,25 +8941,25 @@
       <c r="AA87" s="154"/>
       <c r="AB87" s="154"/>
       <c r="AC87" s="154"/>
-      <c r="AD87" s="359" t="s">
+      <c r="AD87" s="360" t="s">
         <v>137</v>
       </c>
-      <c r="AE87" s="360"/>
-      <c r="AF87" s="361"/>
-      <c r="AG87" s="359"/>
-      <c r="AH87" s="360"/>
-      <c r="AI87" s="361"/>
-      <c r="AJ87" s="362"/>
-      <c r="AK87" s="363"/>
-      <c r="AL87" s="363"/>
-      <c r="AM87" s="363"/>
-      <c r="AN87" s="363"/>
-      <c r="AO87" s="363"/>
-      <c r="AP87" s="363"/>
-      <c r="AQ87" s="363"/>
-      <c r="AR87" s="363"/>
-      <c r="AS87" s="363"/>
-      <c r="AT87" s="364"/>
+      <c r="AE87" s="361"/>
+      <c r="AF87" s="362"/>
+      <c r="AG87" s="360"/>
+      <c r="AH87" s="361"/>
+      <c r="AI87" s="362"/>
+      <c r="AJ87" s="363"/>
+      <c r="AK87" s="364"/>
+      <c r="AL87" s="364"/>
+      <c r="AM87" s="364"/>
+      <c r="AN87" s="364"/>
+      <c r="AO87" s="364"/>
+      <c r="AP87" s="364"/>
+      <c r="AQ87" s="364"/>
+      <c r="AR87" s="364"/>
+      <c r="AS87" s="364"/>
+      <c r="AT87" s="365"/>
       <c r="AU87" s="14"/>
     </row>
     <row r="88" spans="1:47" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -8994,25 +8998,25 @@
       <c r="AA88" s="154"/>
       <c r="AB88" s="154"/>
       <c r="AC88" s="154"/>
-      <c r="AD88" s="359"/>
-      <c r="AE88" s="360"/>
-      <c r="AF88" s="361"/>
-      <c r="AG88" s="359"/>
-      <c r="AH88" s="360"/>
-      <c r="AI88" s="361"/>
-      <c r="AJ88" s="365" t="s">
+      <c r="AD88" s="360"/>
+      <c r="AE88" s="361"/>
+      <c r="AF88" s="362"/>
+      <c r="AG88" s="360"/>
+      <c r="AH88" s="361"/>
+      <c r="AI88" s="362"/>
+      <c r="AJ88" s="366" t="s">
         <v>139</v>
       </c>
-      <c r="AK88" s="366"/>
-      <c r="AL88" s="366"/>
-      <c r="AM88" s="366"/>
-      <c r="AN88" s="366"/>
-      <c r="AO88" s="366"/>
-      <c r="AP88" s="366"/>
-      <c r="AQ88" s="366"/>
-      <c r="AR88" s="366"/>
-      <c r="AS88" s="366"/>
-      <c r="AT88" s="367"/>
+      <c r="AK88" s="367"/>
+      <c r="AL88" s="367"/>
+      <c r="AM88" s="367"/>
+      <c r="AN88" s="367"/>
+      <c r="AO88" s="367"/>
+      <c r="AP88" s="367"/>
+      <c r="AQ88" s="367"/>
+      <c r="AR88" s="367"/>
+      <c r="AS88" s="367"/>
+      <c r="AT88" s="368"/>
       <c r="AU88" s="14"/>
     </row>
     <row r="89" spans="1:47" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -9049,125 +9053,125 @@
       <c r="AA89" s="154"/>
       <c r="AB89" s="154"/>
       <c r="AC89" s="154"/>
-      <c r="AD89" s="359" t="s">
+      <c r="AD89" s="360" t="s">
         <v>137</v>
       </c>
-      <c r="AE89" s="360"/>
-      <c r="AF89" s="361"/>
-      <c r="AG89" s="359"/>
-      <c r="AH89" s="360"/>
-      <c r="AI89" s="361"/>
-      <c r="AJ89" s="362"/>
-      <c r="AK89" s="363"/>
-      <c r="AL89" s="363"/>
-      <c r="AM89" s="363"/>
-      <c r="AN89" s="363"/>
-      <c r="AO89" s="363"/>
-      <c r="AP89" s="363"/>
-      <c r="AQ89" s="363"/>
-      <c r="AR89" s="363"/>
-      <c r="AS89" s="363"/>
-      <c r="AT89" s="364"/>
+      <c r="AE89" s="361"/>
+      <c r="AF89" s="362"/>
+      <c r="AG89" s="360"/>
+      <c r="AH89" s="361"/>
+      <c r="AI89" s="362"/>
+      <c r="AJ89" s="363"/>
+      <c r="AK89" s="364"/>
+      <c r="AL89" s="364"/>
+      <c r="AM89" s="364"/>
+      <c r="AN89" s="364"/>
+      <c r="AO89" s="364"/>
+      <c r="AP89" s="364"/>
+      <c r="AQ89" s="364"/>
+      <c r="AR89" s="364"/>
+      <c r="AS89" s="364"/>
+      <c r="AT89" s="365"/>
       <c r="AU89" s="14"/>
     </row>
     <row r="90" spans="1:47" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A90" s="13"/>
-      <c r="B90" s="358" t="s">
+      <c r="B90" s="359" t="s">
         <v>79</v>
       </c>
-      <c r="C90" s="358"/>
-      <c r="D90" s="358"/>
-      <c r="E90" s="358"/>
-      <c r="F90" s="358"/>
-      <c r="G90" s="358"/>
-      <c r="H90" s="358"/>
-      <c r="I90" s="358"/>
-      <c r="J90" s="358"/>
-      <c r="K90" s="358"/>
-      <c r="L90" s="358"/>
-      <c r="M90" s="358"/>
-      <c r="N90" s="358"/>
-      <c r="O90" s="358"/>
-      <c r="P90" s="358"/>
-      <c r="Q90" s="358"/>
-      <c r="R90" s="358"/>
-      <c r="S90" s="358"/>
-      <c r="T90" s="358"/>
-      <c r="U90" s="358"/>
-      <c r="V90" s="358"/>
-      <c r="W90" s="358"/>
-      <c r="X90" s="358"/>
-      <c r="Y90" s="358"/>
-      <c r="Z90" s="358"/>
-      <c r="AA90" s="358"/>
-      <c r="AB90" s="358"/>
-      <c r="AC90" s="358"/>
-      <c r="AD90" s="358"/>
-      <c r="AE90" s="358"/>
-      <c r="AF90" s="358"/>
-      <c r="AG90" s="358"/>
-      <c r="AH90" s="358"/>
-      <c r="AI90" s="358"/>
-      <c r="AJ90" s="358"/>
-      <c r="AK90" s="358"/>
-      <c r="AL90" s="358"/>
-      <c r="AM90" s="358"/>
-      <c r="AN90" s="358"/>
-      <c r="AO90" s="358"/>
-      <c r="AP90" s="358"/>
-      <c r="AQ90" s="358"/>
-      <c r="AR90" s="358"/>
-      <c r="AS90" s="358"/>
-      <c r="AT90" s="358"/>
+      <c r="C90" s="359"/>
+      <c r="D90" s="359"/>
+      <c r="E90" s="359"/>
+      <c r="F90" s="359"/>
+      <c r="G90" s="359"/>
+      <c r="H90" s="359"/>
+      <c r="I90" s="359"/>
+      <c r="J90" s="359"/>
+      <c r="K90" s="359"/>
+      <c r="L90" s="359"/>
+      <c r="M90" s="359"/>
+      <c r="N90" s="359"/>
+      <c r="O90" s="359"/>
+      <c r="P90" s="359"/>
+      <c r="Q90" s="359"/>
+      <c r="R90" s="359"/>
+      <c r="S90" s="359"/>
+      <c r="T90" s="359"/>
+      <c r="U90" s="359"/>
+      <c r="V90" s="359"/>
+      <c r="W90" s="359"/>
+      <c r="X90" s="359"/>
+      <c r="Y90" s="359"/>
+      <c r="Z90" s="359"/>
+      <c r="AA90" s="359"/>
+      <c r="AB90" s="359"/>
+      <c r="AC90" s="359"/>
+      <c r="AD90" s="359"/>
+      <c r="AE90" s="359"/>
+      <c r="AF90" s="359"/>
+      <c r="AG90" s="359"/>
+      <c r="AH90" s="359"/>
+      <c r="AI90" s="359"/>
+      <c r="AJ90" s="359"/>
+      <c r="AK90" s="359"/>
+      <c r="AL90" s="359"/>
+      <c r="AM90" s="359"/>
+      <c r="AN90" s="359"/>
+      <c r="AO90" s="359"/>
+      <c r="AP90" s="359"/>
+      <c r="AQ90" s="359"/>
+      <c r="AR90" s="359"/>
+      <c r="AS90" s="359"/>
+      <c r="AT90" s="359"/>
       <c r="AU90" s="14"/>
     </row>
     <row r="91" spans="1:47" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A91" s="13"/>
-      <c r="B91" s="355"/>
-      <c r="C91" s="356"/>
-      <c r="D91" s="356"/>
-      <c r="E91" s="356"/>
-      <c r="F91" s="356"/>
-      <c r="G91" s="356"/>
-      <c r="H91" s="356"/>
-      <c r="I91" s="356"/>
-      <c r="J91" s="356"/>
-      <c r="K91" s="356"/>
-      <c r="L91" s="356"/>
-      <c r="M91" s="356"/>
-      <c r="N91" s="356"/>
-      <c r="O91" s="356"/>
-      <c r="P91" s="356"/>
-      <c r="Q91" s="356"/>
-      <c r="R91" s="356"/>
-      <c r="S91" s="356"/>
-      <c r="T91" s="356"/>
-      <c r="U91" s="356"/>
-      <c r="V91" s="356"/>
-      <c r="W91" s="356"/>
-      <c r="X91" s="356"/>
-      <c r="Y91" s="356"/>
-      <c r="Z91" s="356"/>
-      <c r="AA91" s="356"/>
-      <c r="AB91" s="356"/>
-      <c r="AC91" s="356"/>
-      <c r="AD91" s="356"/>
-      <c r="AE91" s="356"/>
-      <c r="AF91" s="356"/>
-      <c r="AG91" s="356"/>
-      <c r="AH91" s="356"/>
-      <c r="AI91" s="356"/>
-      <c r="AJ91" s="356"/>
-      <c r="AK91" s="356"/>
-      <c r="AL91" s="356"/>
-      <c r="AM91" s="356"/>
-      <c r="AN91" s="356"/>
-      <c r="AO91" s="356"/>
-      <c r="AP91" s="356"/>
-      <c r="AQ91" s="356"/>
-      <c r="AR91" s="356"/>
-      <c r="AS91" s="356"/>
-      <c r="AT91" s="357"/>
+      <c r="B91" s="356"/>
+      <c r="C91" s="357"/>
+      <c r="D91" s="357"/>
+      <c r="E91" s="357"/>
+      <c r="F91" s="357"/>
+      <c r="G91" s="357"/>
+      <c r="H91" s="357"/>
+      <c r="I91" s="357"/>
+      <c r="J91" s="357"/>
+      <c r="K91" s="357"/>
+      <c r="L91" s="357"/>
+      <c r="M91" s="357"/>
+      <c r="N91" s="357"/>
+      <c r="O91" s="357"/>
+      <c r="P91" s="357"/>
+      <c r="Q91" s="357"/>
+      <c r="R91" s="357"/>
+      <c r="S91" s="357"/>
+      <c r="T91" s="357"/>
+      <c r="U91" s="357"/>
+      <c r="V91" s="357"/>
+      <c r="W91" s="357"/>
+      <c r="X91" s="357"/>
+      <c r="Y91" s="357"/>
+      <c r="Z91" s="357"/>
+      <c r="AA91" s="357"/>
+      <c r="AB91" s="357"/>
+      <c r="AC91" s="357"/>
+      <c r="AD91" s="357"/>
+      <c r="AE91" s="357"/>
+      <c r="AF91" s="357"/>
+      <c r="AG91" s="357"/>
+      <c r="AH91" s="357"/>
+      <c r="AI91" s="357"/>
+      <c r="AJ91" s="357"/>
+      <c r="AK91" s="357"/>
+      <c r="AL91" s="357"/>
+      <c r="AM91" s="357"/>
+      <c r="AN91" s="357"/>
+      <c r="AO91" s="357"/>
+      <c r="AP91" s="357"/>
+      <c r="AQ91" s="357"/>
+      <c r="AR91" s="357"/>
+      <c r="AS91" s="357"/>
+      <c r="AT91" s="358"/>
       <c r="AU91" s="14"/>
     </row>
     <row r="92" spans="1:47" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -9270,53 +9274,53 @@
     </row>
     <row r="94" spans="1:47" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="13"/>
-      <c r="B94" s="399" t="s">
+      <c r="B94" s="400" t="s">
         <v>77</v>
       </c>
-      <c r="C94" s="399"/>
-      <c r="D94" s="399"/>
-      <c r="E94" s="399"/>
-      <c r="F94" s="399"/>
-      <c r="G94" s="399"/>
-      <c r="H94" s="399"/>
-      <c r="I94" s="399"/>
-      <c r="J94" s="399"/>
-      <c r="K94" s="399"/>
-      <c r="L94" s="399"/>
-      <c r="M94" s="399"/>
-      <c r="N94" s="399"/>
-      <c r="O94" s="399"/>
-      <c r="P94" s="399"/>
-      <c r="Q94" s="399"/>
-      <c r="R94" s="399"/>
-      <c r="S94" s="399"/>
-      <c r="T94" s="399"/>
-      <c r="U94" s="399"/>
-      <c r="V94" s="399"/>
-      <c r="W94" s="399"/>
-      <c r="X94" s="399"/>
-      <c r="Y94" s="399"/>
-      <c r="Z94" s="399"/>
-      <c r="AA94" s="399"/>
-      <c r="AB94" s="399"/>
-      <c r="AC94" s="399"/>
-      <c r="AD94" s="399"/>
-      <c r="AE94" s="399"/>
-      <c r="AF94" s="399"/>
-      <c r="AG94" s="399"/>
-      <c r="AH94" s="399"/>
-      <c r="AI94" s="399"/>
-      <c r="AJ94" s="399"/>
-      <c r="AK94" s="399"/>
-      <c r="AL94" s="399"/>
-      <c r="AM94" s="399"/>
-      <c r="AN94" s="399"/>
-      <c r="AO94" s="399"/>
-      <c r="AP94" s="399"/>
-      <c r="AQ94" s="399"/>
-      <c r="AR94" s="399"/>
-      <c r="AS94" s="399"/>
-      <c r="AT94" s="399"/>
+      <c r="C94" s="400"/>
+      <c r="D94" s="400"/>
+      <c r="E94" s="400"/>
+      <c r="F94" s="400"/>
+      <c r="G94" s="400"/>
+      <c r="H94" s="400"/>
+      <c r="I94" s="400"/>
+      <c r="J94" s="400"/>
+      <c r="K94" s="400"/>
+      <c r="L94" s="400"/>
+      <c r="M94" s="400"/>
+      <c r="N94" s="400"/>
+      <c r="O94" s="400"/>
+      <c r="P94" s="400"/>
+      <c r="Q94" s="400"/>
+      <c r="R94" s="400"/>
+      <c r="S94" s="400"/>
+      <c r="T94" s="400"/>
+      <c r="U94" s="400"/>
+      <c r="V94" s="400"/>
+      <c r="W94" s="400"/>
+      <c r="X94" s="400"/>
+      <c r="Y94" s="400"/>
+      <c r="Z94" s="400"/>
+      <c r="AA94" s="400"/>
+      <c r="AB94" s="400"/>
+      <c r="AC94" s="400"/>
+      <c r="AD94" s="400"/>
+      <c r="AE94" s="400"/>
+      <c r="AF94" s="400"/>
+      <c r="AG94" s="400"/>
+      <c r="AH94" s="400"/>
+      <c r="AI94" s="400"/>
+      <c r="AJ94" s="400"/>
+      <c r="AK94" s="400"/>
+      <c r="AL94" s="400"/>
+      <c r="AM94" s="400"/>
+      <c r="AN94" s="400"/>
+      <c r="AO94" s="400"/>
+      <c r="AP94" s="400"/>
+      <c r="AQ94" s="400"/>
+      <c r="AR94" s="400"/>
+      <c r="AS94" s="400"/>
+      <c r="AT94" s="400"/>
       <c r="AU94" s="14"/>
     </row>
     <row r="95" spans="1:47" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -9666,51 +9670,51 @@
     </row>
     <row r="102" spans="1:47" ht="47.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A102" s="13"/>
-      <c r="B102" s="355"/>
-      <c r="C102" s="356"/>
-      <c r="D102" s="356"/>
-      <c r="E102" s="356"/>
-      <c r="F102" s="356"/>
-      <c r="G102" s="356"/>
-      <c r="H102" s="356"/>
-      <c r="I102" s="356"/>
-      <c r="J102" s="356"/>
-      <c r="K102" s="356"/>
-      <c r="L102" s="356"/>
-      <c r="M102" s="356"/>
-      <c r="N102" s="356"/>
-      <c r="O102" s="356"/>
-      <c r="P102" s="356"/>
-      <c r="Q102" s="356"/>
-      <c r="R102" s="356"/>
-      <c r="S102" s="356"/>
-      <c r="T102" s="356"/>
-      <c r="U102" s="356"/>
-      <c r="V102" s="356"/>
-      <c r="W102" s="356"/>
-      <c r="X102" s="356"/>
-      <c r="Y102" s="356"/>
-      <c r="Z102" s="356"/>
-      <c r="AA102" s="356"/>
-      <c r="AB102" s="356"/>
-      <c r="AC102" s="356"/>
-      <c r="AD102" s="356"/>
-      <c r="AE102" s="356"/>
-      <c r="AF102" s="356"/>
-      <c r="AG102" s="356"/>
-      <c r="AH102" s="356"/>
-      <c r="AI102" s="356"/>
-      <c r="AJ102" s="356"/>
-      <c r="AK102" s="356"/>
-      <c r="AL102" s="356"/>
-      <c r="AM102" s="356"/>
-      <c r="AN102" s="356"/>
-      <c r="AO102" s="356"/>
-      <c r="AP102" s="356"/>
-      <c r="AQ102" s="356"/>
-      <c r="AR102" s="356"/>
-      <c r="AS102" s="356"/>
-      <c r="AT102" s="357"/>
+      <c r="B102" s="356"/>
+      <c r="C102" s="357"/>
+      <c r="D102" s="357"/>
+      <c r="E102" s="357"/>
+      <c r="F102" s="357"/>
+      <c r="G102" s="357"/>
+      <c r="H102" s="357"/>
+      <c r="I102" s="357"/>
+      <c r="J102" s="357"/>
+      <c r="K102" s="357"/>
+      <c r="L102" s="357"/>
+      <c r="M102" s="357"/>
+      <c r="N102" s="357"/>
+      <c r="O102" s="357"/>
+      <c r="P102" s="357"/>
+      <c r="Q102" s="357"/>
+      <c r="R102" s="357"/>
+      <c r="S102" s="357"/>
+      <c r="T102" s="357"/>
+      <c r="U102" s="357"/>
+      <c r="V102" s="357"/>
+      <c r="W102" s="357"/>
+      <c r="X102" s="357"/>
+      <c r="Y102" s="357"/>
+      <c r="Z102" s="357"/>
+      <c r="AA102" s="357"/>
+      <c r="AB102" s="357"/>
+      <c r="AC102" s="357"/>
+      <c r="AD102" s="357"/>
+      <c r="AE102" s="357"/>
+      <c r="AF102" s="357"/>
+      <c r="AG102" s="357"/>
+      <c r="AH102" s="357"/>
+      <c r="AI102" s="357"/>
+      <c r="AJ102" s="357"/>
+      <c r="AK102" s="357"/>
+      <c r="AL102" s="357"/>
+      <c r="AM102" s="357"/>
+      <c r="AN102" s="357"/>
+      <c r="AO102" s="357"/>
+      <c r="AP102" s="357"/>
+      <c r="AQ102" s="357"/>
+      <c r="AR102" s="357"/>
+      <c r="AS102" s="357"/>
+      <c r="AT102" s="358"/>
       <c r="AU102" s="14"/>
     </row>
     <row r="103" spans="1:47" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -9977,7 +9981,7 @@
       <c r="AQ107" s="105"/>
       <c r="AR107" s="105"/>
       <c r="AS107" s="105"/>
-      <c r="AT107" s="400"/>
+      <c r="AT107" s="401"/>
       <c r="AU107" s="14"/>
     </row>
     <row r="108" spans="1:47" ht="51" customHeight="1" x14ac:dyDescent="0.35">
@@ -9985,13 +9989,13 @@
       <c r="B108" s="54">
         <v>1</v>
       </c>
-      <c r="C108" s="379">
+      <c r="C108" s="380">
         <v>45975</v>
       </c>
-      <c r="D108" s="379"/>
-      <c r="E108" s="379"/>
-      <c r="F108" s="379"/>
-      <c r="G108" s="379"/>
+      <c r="D108" s="380"/>
+      <c r="E108" s="380"/>
+      <c r="F108" s="380"/>
+      <c r="G108" s="380"/>
       <c r="H108" s="108" t="s">
         <v>135</v>
       </c>
@@ -10018,33 +10022,33 @@
         <v>9646</v>
       </c>
       <c r="W108" s="108"/>
-      <c r="X108" s="381" t="s">
+      <c r="X108" s="382" t="s">
         <v>136</v>
       </c>
-      <c r="Y108" s="381"/>
-      <c r="Z108" s="381"/>
-      <c r="AA108" s="381"/>
-      <c r="AB108" s="381"/>
-      <c r="AC108" s="381"/>
-      <c r="AD108" s="381"/>
-      <c r="AE108" s="381"/>
-      <c r="AF108" s="381"/>
-      <c r="AG108" s="381"/>
-      <c r="AH108" s="381"/>
-      <c r="AI108" s="381"/>
-      <c r="AJ108" s="381"/>
-      <c r="AK108" s="381"/>
-      <c r="AL108" s="381"/>
-      <c r="AM108" s="381"/>
-      <c r="AN108" s="371">
+      <c r="Y108" s="382"/>
+      <c r="Z108" s="382"/>
+      <c r="AA108" s="382"/>
+      <c r="AB108" s="382"/>
+      <c r="AC108" s="382"/>
+      <c r="AD108" s="382"/>
+      <c r="AE108" s="382"/>
+      <c r="AF108" s="382"/>
+      <c r="AG108" s="382"/>
+      <c r="AH108" s="382"/>
+      <c r="AI108" s="382"/>
+      <c r="AJ108" s="382"/>
+      <c r="AK108" s="382"/>
+      <c r="AL108" s="382"/>
+      <c r="AM108" s="382"/>
+      <c r="AN108" s="372">
         <v>27331418.760000002</v>
       </c>
-      <c r="AO108" s="371"/>
-      <c r="AP108" s="371"/>
-      <c r="AQ108" s="371"/>
-      <c r="AR108" s="371"/>
-      <c r="AS108" s="371"/>
-      <c r="AT108" s="372"/>
+      <c r="AO108" s="372"/>
+      <c r="AP108" s="372"/>
+      <c r="AQ108" s="372"/>
+      <c r="AR108" s="372"/>
+      <c r="AS108" s="372"/>
+      <c r="AT108" s="373"/>
       <c r="AU108" s="14"/>
     </row>
     <row r="109" spans="1:47" ht="13" x14ac:dyDescent="0.35">
@@ -10205,43 +10209,43 @@
       <c r="B112" s="40">
         <v>5</v>
       </c>
-      <c r="C112" s="376"/>
-      <c r="D112" s="376"/>
-      <c r="E112" s="376"/>
-      <c r="F112" s="376"/>
-      <c r="G112" s="376"/>
-      <c r="H112" s="376"/>
-      <c r="I112" s="376"/>
-      <c r="J112" s="376"/>
-      <c r="K112" s="376"/>
-      <c r="L112" s="376"/>
-      <c r="M112" s="377"/>
-      <c r="N112" s="377"/>
-      <c r="O112" s="377"/>
-      <c r="P112" s="377"/>
-      <c r="Q112" s="377"/>
-      <c r="R112" s="377"/>
-      <c r="S112" s="377"/>
-      <c r="T112" s="377"/>
-      <c r="U112" s="377"/>
-      <c r="V112" s="377"/>
-      <c r="W112" s="377"/>
-      <c r="X112" s="376"/>
-      <c r="Y112" s="376"/>
-      <c r="Z112" s="376"/>
-      <c r="AA112" s="376"/>
-      <c r="AB112" s="376"/>
-      <c r="AC112" s="376"/>
-      <c r="AD112" s="376"/>
-      <c r="AE112" s="376"/>
-      <c r="AF112" s="376"/>
-      <c r="AG112" s="376"/>
-      <c r="AH112" s="376"/>
-      <c r="AI112" s="376"/>
-      <c r="AJ112" s="376"/>
-      <c r="AK112" s="376"/>
-      <c r="AL112" s="376"/>
-      <c r="AM112" s="376"/>
+      <c r="C112" s="377"/>
+      <c r="D112" s="377"/>
+      <c r="E112" s="377"/>
+      <c r="F112" s="377"/>
+      <c r="G112" s="377"/>
+      <c r="H112" s="377"/>
+      <c r="I112" s="377"/>
+      <c r="J112" s="377"/>
+      <c r="K112" s="377"/>
+      <c r="L112" s="377"/>
+      <c r="M112" s="378"/>
+      <c r="N112" s="378"/>
+      <c r="O112" s="378"/>
+      <c r="P112" s="378"/>
+      <c r="Q112" s="378"/>
+      <c r="R112" s="378"/>
+      <c r="S112" s="378"/>
+      <c r="T112" s="378"/>
+      <c r="U112" s="378"/>
+      <c r="V112" s="378"/>
+      <c r="W112" s="378"/>
+      <c r="X112" s="377"/>
+      <c r="Y112" s="377"/>
+      <c r="Z112" s="377"/>
+      <c r="AA112" s="377"/>
+      <c r="AB112" s="377"/>
+      <c r="AC112" s="377"/>
+      <c r="AD112" s="377"/>
+      <c r="AE112" s="377"/>
+      <c r="AF112" s="377"/>
+      <c r="AG112" s="377"/>
+      <c r="AH112" s="377"/>
+      <c r="AI112" s="377"/>
+      <c r="AJ112" s="377"/>
+      <c r="AK112" s="377"/>
+      <c r="AL112" s="377"/>
+      <c r="AM112" s="377"/>
       <c r="AN112" s="201"/>
       <c r="AO112" s="201"/>
       <c r="AP112" s="201"/>
@@ -10293,16 +10297,16 @@
       <c r="AM113" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="AN113" s="373">
+      <c r="AN113" s="374">
         <f>SUM(AN108:AT112)</f>
         <v>27331418.760000002</v>
       </c>
-      <c r="AO113" s="374"/>
-      <c r="AP113" s="374"/>
-      <c r="AQ113" s="374"/>
-      <c r="AR113" s="374"/>
-      <c r="AS113" s="374"/>
-      <c r="AT113" s="375"/>
+      <c r="AO113" s="375"/>
+      <c r="AP113" s="375"/>
+      <c r="AQ113" s="375"/>
+      <c r="AR113" s="375"/>
+      <c r="AS113" s="375"/>
+      <c r="AT113" s="376"/>
       <c r="AU113" s="14"/>
     </row>
     <row r="114" spans="1:52" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -10339,19 +10343,19 @@
       <c r="AE114" s="2"/>
       <c r="AF114" s="2"/>
       <c r="AG114" s="2"/>
-      <c r="AH114" s="378"/>
-      <c r="AI114" s="378"/>
-      <c r="AJ114" s="378"/>
-      <c r="AK114" s="378"/>
-      <c r="AL114" s="378"/>
-      <c r="AM114" s="378"/>
-      <c r="AN114" s="378"/>
-      <c r="AO114" s="378"/>
-      <c r="AP114" s="378"/>
-      <c r="AQ114" s="378"/>
-      <c r="AR114" s="378"/>
-      <c r="AS114" s="378"/>
-      <c r="AT114" s="378"/>
+      <c r="AH114" s="379"/>
+      <c r="AI114" s="379"/>
+      <c r="AJ114" s="379"/>
+      <c r="AK114" s="379"/>
+      <c r="AL114" s="379"/>
+      <c r="AM114" s="379"/>
+      <c r="AN114" s="379"/>
+      <c r="AO114" s="379"/>
+      <c r="AP114" s="379"/>
+      <c r="AQ114" s="379"/>
+      <c r="AR114" s="379"/>
+      <c r="AS114" s="379"/>
+      <c r="AT114" s="379"/>
       <c r="AU114" s="14"/>
     </row>
     <row r="115" spans="1:52" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -10388,19 +10392,19 @@
       <c r="AE115" s="2"/>
       <c r="AF115" s="2"/>
       <c r="AG115" s="2"/>
-      <c r="AH115" s="378"/>
-      <c r="AI115" s="378"/>
-      <c r="AJ115" s="378"/>
-      <c r="AK115" s="378"/>
-      <c r="AL115" s="378"/>
-      <c r="AM115" s="378"/>
-      <c r="AN115" s="378"/>
-      <c r="AO115" s="378"/>
-      <c r="AP115" s="378"/>
-      <c r="AQ115" s="378"/>
-      <c r="AR115" s="378"/>
-      <c r="AS115" s="378"/>
-      <c r="AT115" s="378"/>
+      <c r="AH115" s="379"/>
+      <c r="AI115" s="379"/>
+      <c r="AJ115" s="379"/>
+      <c r="AK115" s="379"/>
+      <c r="AL115" s="379"/>
+      <c r="AM115" s="379"/>
+      <c r="AN115" s="379"/>
+      <c r="AO115" s="379"/>
+      <c r="AP115" s="379"/>
+      <c r="AQ115" s="379"/>
+      <c r="AR115" s="379"/>
+      <c r="AS115" s="379"/>
+      <c r="AT115" s="379"/>
       <c r="AU115" s="14"/>
     </row>
     <row r="116" spans="1:52" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -10473,25 +10477,25 @@
       <c r="J117" s="207"/>
       <c r="K117" s="207"/>
       <c r="L117" s="207"/>
-      <c r="M117" s="386" t="s">
+      <c r="M117" s="387" t="s">
         <v>48</v>
       </c>
-      <c r="N117" s="386"/>
-      <c r="O117" s="386"/>
-      <c r="P117" s="386" t="s">
+      <c r="N117" s="387"/>
+      <c r="O117" s="387"/>
+      <c r="P117" s="387" t="s">
         <v>59</v>
       </c>
-      <c r="Q117" s="386"/>
-      <c r="R117" s="386"/>
-      <c r="S117" s="386" t="s">
+      <c r="Q117" s="387"/>
+      <c r="R117" s="387"/>
+      <c r="S117" s="387" t="s">
         <v>50</v>
       </c>
-      <c r="T117" s="386"/>
-      <c r="U117" s="386"/>
-      <c r="V117" s="386" t="s">
+      <c r="T117" s="387"/>
+      <c r="U117" s="387"/>
+      <c r="V117" s="387" t="s">
         <v>60</v>
       </c>
-      <c r="W117" s="386"/>
+      <c r="W117" s="387"/>
       <c r="X117" s="207" t="s">
         <v>51</v>
       </c>
@@ -10538,7 +10542,7 @@
       <c r="F118" s="179"/>
       <c r="G118" s="179"/>
       <c r="H118" s="176" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I118" s="176"/>
       <c r="J118" s="176"/>
@@ -10563,33 +10567,33 @@
         <v>9646</v>
       </c>
       <c r="W118" s="176"/>
-      <c r="X118" s="383" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y118" s="383"/>
-      <c r="Z118" s="383"/>
-      <c r="AA118" s="383"/>
-      <c r="AB118" s="383"/>
-      <c r="AC118" s="383"/>
-      <c r="AD118" s="383"/>
-      <c r="AE118" s="383"/>
-      <c r="AF118" s="383"/>
-      <c r="AG118" s="383"/>
-      <c r="AH118" s="383"/>
-      <c r="AI118" s="383"/>
-      <c r="AJ118" s="383"/>
-      <c r="AK118" s="383"/>
-      <c r="AL118" s="383"/>
-      <c r="AM118" s="383"/>
-      <c r="AN118" s="397">
-        <v>22200000</v>
-      </c>
-      <c r="AO118" s="397"/>
-      <c r="AP118" s="397"/>
-      <c r="AQ118" s="397"/>
-      <c r="AR118" s="397"/>
-      <c r="AS118" s="397"/>
-      <c r="AT118" s="398"/>
+      <c r="X118" s="384" t="s">
+        <v>144</v>
+      </c>
+      <c r="Y118" s="384"/>
+      <c r="Z118" s="384"/>
+      <c r="AA118" s="384"/>
+      <c r="AB118" s="384"/>
+      <c r="AC118" s="384"/>
+      <c r="AD118" s="384"/>
+      <c r="AE118" s="384"/>
+      <c r="AF118" s="384"/>
+      <c r="AG118" s="384"/>
+      <c r="AH118" s="384"/>
+      <c r="AI118" s="384"/>
+      <c r="AJ118" s="384"/>
+      <c r="AK118" s="384"/>
+      <c r="AL118" s="384"/>
+      <c r="AM118" s="384"/>
+      <c r="AN118" s="398">
+        <v>900000000</v>
+      </c>
+      <c r="AO118" s="398"/>
+      <c r="AP118" s="398"/>
+      <c r="AQ118" s="398"/>
+      <c r="AR118" s="398"/>
+      <c r="AS118" s="398"/>
+      <c r="AT118" s="399"/>
       <c r="AU118" s="62"/>
       <c r="AZ118" s="94">
         <v>59200000</v>
@@ -10635,7 +10639,7 @@
       <c r="AK119" s="71"/>
       <c r="AL119" s="71"/>
       <c r="AM119" s="71"/>
-      <c r="AN119" s="97"/>
+      <c r="AN119" s="415"/>
       <c r="AO119" s="97"/>
       <c r="AP119" s="97"/>
       <c r="AQ119" s="97"/>
@@ -10650,53 +10654,53 @@
     </row>
     <row r="120" spans="1:52" s="63" customFormat="1" ht="12.65" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A120" s="59"/>
-      <c r="B120" s="393" t="s">
+      <c r="B120" s="394" t="s">
         <v>94</v>
       </c>
-      <c r="C120" s="393"/>
-      <c r="D120" s="393"/>
-      <c r="E120" s="393"/>
-      <c r="F120" s="393"/>
-      <c r="G120" s="393"/>
-      <c r="H120" s="393"/>
-      <c r="I120" s="393"/>
-      <c r="J120" s="393"/>
-      <c r="K120" s="393"/>
-      <c r="L120" s="393"/>
-      <c r="M120" s="393"/>
-      <c r="N120" s="393"/>
-      <c r="O120" s="393"/>
-      <c r="P120" s="393"/>
-      <c r="Q120" s="393"/>
-      <c r="R120" s="393"/>
-      <c r="S120" s="393"/>
-      <c r="T120" s="393"/>
-      <c r="U120" s="393"/>
-      <c r="V120" s="393"/>
-      <c r="W120" s="393"/>
-      <c r="X120" s="393"/>
-      <c r="Y120" s="393"/>
-      <c r="Z120" s="393"/>
-      <c r="AA120" s="393"/>
-      <c r="AB120" s="393"/>
-      <c r="AC120" s="393"/>
-      <c r="AD120" s="393"/>
-      <c r="AE120" s="393"/>
-      <c r="AF120" s="393"/>
-      <c r="AG120" s="393"/>
-      <c r="AH120" s="393"/>
-      <c r="AI120" s="393"/>
-      <c r="AJ120" s="393"/>
-      <c r="AK120" s="393"/>
-      <c r="AL120" s="393"/>
-      <c r="AM120" s="393"/>
-      <c r="AN120" s="393"/>
-      <c r="AO120" s="393"/>
-      <c r="AP120" s="393"/>
-      <c r="AQ120" s="393"/>
-      <c r="AR120" s="393"/>
-      <c r="AS120" s="393"/>
-      <c r="AT120" s="393"/>
+      <c r="C120" s="394"/>
+      <c r="D120" s="394"/>
+      <c r="E120" s="394"/>
+      <c r="F120" s="394"/>
+      <c r="G120" s="394"/>
+      <c r="H120" s="394"/>
+      <c r="I120" s="394"/>
+      <c r="J120" s="394"/>
+      <c r="K120" s="394"/>
+      <c r="L120" s="394"/>
+      <c r="M120" s="394"/>
+      <c r="N120" s="394"/>
+      <c r="O120" s="394"/>
+      <c r="P120" s="394"/>
+      <c r="Q120" s="394"/>
+      <c r="R120" s="394"/>
+      <c r="S120" s="394"/>
+      <c r="T120" s="394"/>
+      <c r="U120" s="394"/>
+      <c r="V120" s="394"/>
+      <c r="W120" s="394"/>
+      <c r="X120" s="394"/>
+      <c r="Y120" s="394"/>
+      <c r="Z120" s="394"/>
+      <c r="AA120" s="394"/>
+      <c r="AB120" s="394"/>
+      <c r="AC120" s="394"/>
+      <c r="AD120" s="394"/>
+      <c r="AE120" s="394"/>
+      <c r="AF120" s="394"/>
+      <c r="AG120" s="394"/>
+      <c r="AH120" s="394"/>
+      <c r="AI120" s="394"/>
+      <c r="AJ120" s="394"/>
+      <c r="AK120" s="394"/>
+      <c r="AL120" s="394"/>
+      <c r="AM120" s="394"/>
+      <c r="AN120" s="394"/>
+      <c r="AO120" s="394"/>
+      <c r="AP120" s="394"/>
+      <c r="AQ120" s="394"/>
+      <c r="AR120" s="394"/>
+      <c r="AS120" s="394"/>
+      <c r="AT120" s="394"/>
       <c r="AU120" s="62"/>
       <c r="AZ120" s="94"/>
     </row>
@@ -10752,53 +10756,53 @@
     </row>
     <row r="122" spans="1:52" s="63" customFormat="1" ht="28.5" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A122" s="59"/>
-      <c r="B122" s="394" t="s">
+      <c r="B122" s="395" t="s">
         <v>93</v>
       </c>
-      <c r="C122" s="395"/>
-      <c r="D122" s="395"/>
-      <c r="E122" s="395"/>
-      <c r="F122" s="395"/>
-      <c r="G122" s="395"/>
-      <c r="H122" s="395"/>
-      <c r="I122" s="395"/>
-      <c r="J122" s="395"/>
-      <c r="K122" s="395"/>
-      <c r="L122" s="395"/>
-      <c r="M122" s="395"/>
-      <c r="N122" s="395"/>
-      <c r="O122" s="395"/>
-      <c r="P122" s="395"/>
-      <c r="Q122" s="395"/>
-      <c r="R122" s="395"/>
-      <c r="S122" s="395"/>
-      <c r="T122" s="395"/>
-      <c r="U122" s="395"/>
-      <c r="V122" s="395"/>
-      <c r="W122" s="395"/>
-      <c r="X122" s="395"/>
-      <c r="Y122" s="395"/>
-      <c r="Z122" s="395"/>
-      <c r="AA122" s="395"/>
-      <c r="AB122" s="395"/>
-      <c r="AC122" s="395"/>
-      <c r="AD122" s="395"/>
-      <c r="AE122" s="395"/>
-      <c r="AF122" s="395"/>
-      <c r="AG122" s="395"/>
-      <c r="AH122" s="395"/>
-      <c r="AI122" s="395"/>
-      <c r="AJ122" s="395"/>
-      <c r="AK122" s="395"/>
-      <c r="AL122" s="395"/>
-      <c r="AM122" s="395"/>
-      <c r="AN122" s="395"/>
-      <c r="AO122" s="395"/>
-      <c r="AP122" s="395"/>
-      <c r="AQ122" s="395"/>
-      <c r="AR122" s="395"/>
-      <c r="AS122" s="395"/>
-      <c r="AT122" s="396"/>
+      <c r="C122" s="396"/>
+      <c r="D122" s="396"/>
+      <c r="E122" s="396"/>
+      <c r="F122" s="396"/>
+      <c r="G122" s="396"/>
+      <c r="H122" s="396"/>
+      <c r="I122" s="396"/>
+      <c r="J122" s="396"/>
+      <c r="K122" s="396"/>
+      <c r="L122" s="396"/>
+      <c r="M122" s="396"/>
+      <c r="N122" s="396"/>
+      <c r="O122" s="396"/>
+      <c r="P122" s="396"/>
+      <c r="Q122" s="396"/>
+      <c r="R122" s="396"/>
+      <c r="S122" s="396"/>
+      <c r="T122" s="396"/>
+      <c r="U122" s="396"/>
+      <c r="V122" s="396"/>
+      <c r="W122" s="396"/>
+      <c r="X122" s="396"/>
+      <c r="Y122" s="396"/>
+      <c r="Z122" s="396"/>
+      <c r="AA122" s="396"/>
+      <c r="AB122" s="396"/>
+      <c r="AC122" s="396"/>
+      <c r="AD122" s="396"/>
+      <c r="AE122" s="396"/>
+      <c r="AF122" s="396"/>
+      <c r="AG122" s="396"/>
+      <c r="AH122" s="396"/>
+      <c r="AI122" s="396"/>
+      <c r="AJ122" s="396"/>
+      <c r="AK122" s="396"/>
+      <c r="AL122" s="396"/>
+      <c r="AM122" s="396"/>
+      <c r="AN122" s="396"/>
+      <c r="AO122" s="396"/>
+      <c r="AP122" s="396"/>
+      <c r="AQ122" s="396"/>
+      <c r="AR122" s="396"/>
+      <c r="AS122" s="396"/>
+      <c r="AT122" s="397"/>
       <c r="AU122" s="62"/>
       <c r="AZ122" s="94"/>
     </row>
@@ -10861,12 +10865,12 @@
       <c r="F124" s="60"/>
       <c r="G124" s="60"/>
       <c r="H124" s="101"/>
-      <c r="I124" s="385"/>
-      <c r="J124" s="385"/>
-      <c r="K124" s="385"/>
-      <c r="L124" s="385"/>
-      <c r="M124" s="385"/>
-      <c r="N124" s="385"/>
+      <c r="I124" s="386"/>
+      <c r="J124" s="386"/>
+      <c r="K124" s="386"/>
+      <c r="L124" s="386"/>
+      <c r="M124" s="386"/>
+      <c r="N124" s="386"/>
       <c r="O124" s="61"/>
       <c r="P124" s="61"/>
       <c r="Q124" s="100"/>
@@ -10877,13 +10881,13 @@
       <c r="V124" s="61"/>
       <c r="W124" s="61"/>
       <c r="X124" s="101"/>
-      <c r="Y124" s="385"/>
-      <c r="Z124" s="385"/>
-      <c r="AA124" s="385"/>
-      <c r="AB124" s="385"/>
-      <c r="AC124" s="385"/>
-      <c r="AD124" s="385"/>
-      <c r="AE124" s="385"/>
+      <c r="Y124" s="386"/>
+      <c r="Z124" s="386"/>
+      <c r="AA124" s="386"/>
+      <c r="AB124" s="386"/>
+      <c r="AC124" s="386"/>
+      <c r="AD124" s="386"/>
+      <c r="AE124" s="386"/>
       <c r="AF124" s="100"/>
       <c r="AG124" s="100"/>
       <c r="AH124" s="61"/>
@@ -10894,16 +10898,16 @@
       <c r="AM124" s="101" t="s">
         <v>35</v>
       </c>
-      <c r="AN124" s="390">
+      <c r="AN124" s="391">
         <f>+J37</f>
         <v>476128219</v>
       </c>
-      <c r="AO124" s="391"/>
-      <c r="AP124" s="391"/>
-      <c r="AQ124" s="391"/>
-      <c r="AR124" s="391"/>
-      <c r="AS124" s="391"/>
-      <c r="AT124" s="392"/>
+      <c r="AO124" s="392"/>
+      <c r="AP124" s="392"/>
+      <c r="AQ124" s="392"/>
+      <c r="AR124" s="392"/>
+      <c r="AS124" s="392"/>
+      <c r="AT124" s="393"/>
       <c r="AU124" s="62"/>
       <c r="AZ124" s="94">
         <v>22200000</v>
@@ -10981,16 +10985,16 @@
       <c r="AM126" s="101" t="s">
         <v>36</v>
       </c>
-      <c r="AN126" s="368">
+      <c r="AN126" s="369">
         <f>+AN113</f>
         <v>27331418.760000002</v>
       </c>
-      <c r="AO126" s="369"/>
-      <c r="AP126" s="369"/>
-      <c r="AQ126" s="369"/>
-      <c r="AR126" s="369"/>
-      <c r="AS126" s="369"/>
-      <c r="AT126" s="370"/>
+      <c r="AO126" s="370"/>
+      <c r="AP126" s="370"/>
+      <c r="AQ126" s="370"/>
+      <c r="AR126" s="370"/>
+      <c r="AS126" s="370"/>
+      <c r="AT126" s="371"/>
       <c r="AU126" s="62"/>
       <c r="AZ126" s="94">
         <f>+AZ119-AZ124</f>
@@ -11057,16 +11061,16 @@
       <c r="AM128" s="101" t="s">
         <v>38</v>
       </c>
-      <c r="AN128" s="368">
+      <c r="AN128" s="369">
         <f>SUM(AN118:AT118)</f>
-        <v>22200000</v>
-      </c>
-      <c r="AO128" s="369"/>
-      <c r="AP128" s="369"/>
-      <c r="AQ128" s="369"/>
-      <c r="AR128" s="369"/>
-      <c r="AS128" s="369"/>
-      <c r="AT128" s="370"/>
+        <v>900000000</v>
+      </c>
+      <c r="AO128" s="370"/>
+      <c r="AP128" s="370"/>
+      <c r="AQ128" s="370"/>
+      <c r="AR128" s="370"/>
+      <c r="AS128" s="370"/>
+      <c r="AT128" s="371"/>
       <c r="AU128" s="62"/>
       <c r="AZ128" s="94">
         <f>+AZ126-AZ127</f>
@@ -11120,16 +11124,16 @@
       <c r="AM130" s="101" t="s">
         <v>37</v>
       </c>
-      <c r="AN130" s="368">
+      <c r="AN130" s="369">
         <f>AN124-(AN126+AN128)</f>
-        <v>426596800.24000001</v>
-      </c>
-      <c r="AO130" s="369"/>
-      <c r="AP130" s="369"/>
-      <c r="AQ130" s="369"/>
-      <c r="AR130" s="369"/>
-      <c r="AS130" s="369"/>
-      <c r="AT130" s="370"/>
+        <v>-451203199.75999999</v>
+      </c>
+      <c r="AO130" s="370"/>
+      <c r="AP130" s="370"/>
+      <c r="AQ130" s="370"/>
+      <c r="AR130" s="370"/>
+      <c r="AS130" s="370"/>
+      <c r="AT130" s="371"/>
       <c r="AU130" s="62"/>
       <c r="AZ130" s="103">
         <f>+AN42</f>
@@ -11222,13 +11226,13 @@
       <c r="AM132" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="AN132" s="387"/>
-      <c r="AO132" s="388"/>
-      <c r="AP132" s="388"/>
-      <c r="AQ132" s="388"/>
-      <c r="AR132" s="388"/>
-      <c r="AS132" s="388"/>
-      <c r="AT132" s="389"/>
+      <c r="AN132" s="388"/>
+      <c r="AO132" s="389"/>
+      <c r="AP132" s="389"/>
+      <c r="AQ132" s="389"/>
+      <c r="AR132" s="389"/>
+      <c r="AS132" s="389"/>
+      <c r="AT132" s="390"/>
       <c r="AU132" s="14"/>
       <c r="AZ132" s="56">
         <v>54000000</v>
@@ -11252,21 +11256,21 @@
       <c r="O133" s="19"/>
       <c r="P133" s="19"/>
       <c r="Q133" s="19"/>
-      <c r="AA133" s="380" t="s">
+      <c r="AA133" s="381" t="s">
         <v>97</v>
       </c>
-      <c r="AB133" s="380"/>
-      <c r="AC133" s="380"/>
-      <c r="AD133" s="380"/>
-      <c r="AE133" s="380"/>
-      <c r="AF133" s="380"/>
-      <c r="AG133" s="380"/>
-      <c r="AH133" s="380"/>
-      <c r="AI133" s="380"/>
-      <c r="AJ133" s="380"/>
-      <c r="AK133" s="380"/>
-      <c r="AL133" s="380"/>
-      <c r="AM133" s="380"/>
+      <c r="AB133" s="381"/>
+      <c r="AC133" s="381"/>
+      <c r="AD133" s="381"/>
+      <c r="AE133" s="381"/>
+      <c r="AF133" s="381"/>
+      <c r="AG133" s="381"/>
+      <c r="AH133" s="381"/>
+      <c r="AI133" s="381"/>
+      <c r="AJ133" s="381"/>
+      <c r="AK133" s="381"/>
+      <c r="AL133" s="381"/>
+      <c r="AM133" s="381"/>
       <c r="AU133" s="14"/>
       <c r="AZ133" s="57">
         <f>+AZ131-AZ132</f>
@@ -11292,15 +11296,15 @@
       <c r="AK134" s="2"/>
       <c r="AL134" s="2"/>
       <c r="AM134" s="1"/>
-      <c r="AN134" s="382" t="s">
+      <c r="AN134" s="383" t="s">
         <v>58</v>
       </c>
-      <c r="AO134" s="382"/>
-      <c r="AP134" s="382"/>
-      <c r="AQ134" s="382"/>
-      <c r="AR134" s="382"/>
-      <c r="AS134" s="382"/>
-      <c r="AT134" s="382"/>
+      <c r="AO134" s="383"/>
+      <c r="AP134" s="383"/>
+      <c r="AQ134" s="383"/>
+      <c r="AR134" s="383"/>
+      <c r="AS134" s="383"/>
+      <c r="AT134" s="383"/>
       <c r="AU134" s="14"/>
       <c r="AZ134" s="56">
         <v>29596800</v>
@@ -11320,19 +11324,19 @@
       <c r="I135" s="136"/>
       <c r="J135" s="136"/>
       <c r="K135" s="136"/>
-      <c r="L135" s="384" t="s">
+      <c r="L135" s="385" t="s">
         <v>140</v>
       </c>
-      <c r="M135" s="384"/>
-      <c r="N135" s="384"/>
-      <c r="O135" s="384"/>
-      <c r="P135" s="384"/>
-      <c r="Q135" s="384"/>
-      <c r="R135" s="384"/>
-      <c r="S135" s="384"/>
-      <c r="T135" s="384"/>
-      <c r="U135" s="384"/>
-      <c r="V135" s="384"/>
+      <c r="M135" s="385"/>
+      <c r="N135" s="385"/>
+      <c r="O135" s="385"/>
+      <c r="P135" s="385"/>
+      <c r="Q135" s="385"/>
+      <c r="R135" s="385"/>
+      <c r="S135" s="385"/>
+      <c r="T135" s="385"/>
+      <c r="U135" s="385"/>
+      <c r="V135" s="385"/>
       <c r="W135" s="31"/>
       <c r="X135" s="33" t="s">
         <v>82</v>
@@ -11979,7 +11983,7 @@
         <v>41</v>
       </c>
       <c r="AD148" s="113" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AE148" s="113"/>
       <c r="AF148" s="113"/>

</xml_diff>